<commit_message>
feat: Add SQLite persistence layer for historical deal storage
- Created pipeline/database.py with full CRUD operations
- Integrated as Stage 6 in main.py (non-fatal on error)
- INSERT OR IGNORE prevents re-processing across runs
- Added deals.db to .gitignore (runtime artifact)
</commit_message>
<xml_diff>
--- a/docs/newsletter.xlsx
+++ b/docs/newsletter.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FMCG Deal Intelligence" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FMCG Deal Intelligence'!$A$1:$N$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FMCG Deal Intelligence'!$A$1:$N$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -38,7 +38,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -53,8 +53,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEBEE"/>
-        <bgColor rgb="00FFEBEE"/>
+        <fgColor rgb="00E8F5E9"/>
+        <bgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3E0"/>
+        <bgColor rgb="00FFF3E0"/>
       </patternFill>
     </fill>
   </fills>
@@ -84,13 +90,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -456,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -550,17 +557,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Danone announces $1.6bn acquisition of nutrition drink Huel - Inside FMCG</t>
+          <t>Nestlé Acquires High-End Snack Brand Fireside Foods for $2.1 Billion</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Inside FMCG</t>
+          <t>Reuters</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -570,93 +577,1425 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>$1.6bn</t>
+          <t>$2.1 billion</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Danone</t>
+          <t>Nestlé</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Huel</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
+          <t>Fireside Foods</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Packaged Snacks</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
       <c r="J2" s="2" t="n">
         <v>99</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>75.40000000000001</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Tier 1 — Premier</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQNFF0VjNQeVdlRzUzRzVTODR2eWVhY051M29lNTRYR2Q3Qm5wU2ZDTHZoRWZjNm8wN1R2UW9IZDU2SUxXWDRGXzY2b1VramN5VW5xZ09aTlFObTBITEc5OTJhUFFJZzFYLURmbGtWYkRWNHhPeXl0ZnFkR2xaaVlPZFk0MXRmd3I2alFmUlJFYnFXcG5VMkZ5TjNhNHE?oc=5</t>
+          <t>https://www.reuters.com/business/nestle-acquires-fireside-foods-2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>FMCG stock jumps after NCLT approves merger with Milk Mantra - MSN</t>
+          <t>Unilever Invests $450M in Indian Personal Care Startup GlowNaturals</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>MSN</t>
+          <t>Economic Times</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>Investment</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>$450 million</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Unilever</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>GlowNaturals</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Personal Care</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>97.40000000000001</v>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Tier 1 — Premier</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>https://economictimes.indiatimes.com/unilever-glownaturals-investment</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Marico Picks Up 40% Stake in Vietnamese Coconut Oil Brand CocoViet</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Economic Times</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Investment</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>$35 million</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Marico</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>CocoViet</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Personal Care</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Southeast Asia</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>97.40000000000001</v>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Tier 1 — Premier</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>https://economictimes.indiatimes.com/marico-cocoviet-investment</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Danone Divests North American Yogurt Business to Private Equity Firm Meridian Capital</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Financial Times</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Divestiture</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>$3.8 billion</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Meridian Capital Partners</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Danone's North American yogurt business</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Dairy</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>97.40000000000001</v>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Tier 1 — Premier</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ft.com/content/danone-yogurt-divestiture</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Mondelez International Completes Acquisition of Brazilian Confectionery Group DoceBrasil</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Reuters</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
           <t>M&amp;A</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Milk Mantra</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="n">
-        <v>88</v>
-      </c>
-      <c r="K3" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="L3" s="2" t="n">
-        <v>68.8</v>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNSThvLUYtMmI5VGN2cHNRRG50c09JZkluZVRqVDluYmt4SEJXUnJVSzVnVDVrbFFpb2tmNlBFVmlqSjcwOWVRdGZoZjFYZnRITHNiYlZuWFpZTTJsUkFSNlhFaHc2QWxONEtQUUROWWRFT2YxTGhpR2FBYlBSUTRROV9zb2RwNkJtUWhkQTQxMlhKRVEzLXYxUnk5U2VTNVUzdTlfNmZuMlg2d2o5TWJ0djZn?oc=5</t>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>$1.4 billion</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Mondelez International</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>DoceBrasil</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Confectionery</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>97.40000000000001</v>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Tier 1 — Premier</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reuters.com/business/mondelez-docebrasil-acquisition-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>L'Oréal Acquires Japanese Skincare Brand HadaZen for $900 Million</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Bloomberg</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>$900 million</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>L'Oréal</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>HadaZen</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Cosmetics</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Asia-Pacific</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>97.40000000000001</v>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Tier 1 — Premier</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bloomberg.com/news/loreal-hadazen-acquisition</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>PepsiCo and Britannia Industries Form Joint Venture for Healthy Snacks in India</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Economic Times</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>₹800 crore ($95 million)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>PepsiCo Inc and Britannia Industries</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Packaged Snacks</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>97.40000000000001</v>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>Tier 1 — Premier</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>https://economictimes.indiatimes.com/pepsico-britannia-jv</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Reckitt Benckiser Sells Southeast Asian Fabric Care Division to Henkel for $650M</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Wall Street Journal</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Divestiture</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>$650 million</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Henkel</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Reckitt Benckiser's Southeast Asian fabric care division</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Household Care</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Southeast Asia</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>97.40000000000001</v>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Tier 1 — Premier</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.wsj.com/articles/reckitt-henkel-fabric-care-deal</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Kraft Heinz to Acquire Mexican Condiments Brand SaborRico for $180M</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Reuters</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>$180 million</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Kraft Heinz Company</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>SaborRico</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Condiments &amp; Sauces</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>97.40000000000001</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Tier 1 — Premier</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reuters.com/business/kraft-heinz-saborrico-acquisition</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Estée Lauder Acquires Korean Beauty Brand SeoulGlow in $550M Deal</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Bloomberg</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>$550 million</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Estée Lauder Companies</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>SeoulGlow</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Cosmetics</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Asia-Pacific</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>97.40000000000001</v>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>Tier 1 — Premier</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bloomberg.com/news/estee-lauder-seoulglow</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Dabur India Invests ₹400 Crore in Organic Baby Care Brand TinyOrganics</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Economic Times</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>₹400 crore ($48 million)</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Dabur India</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>TinyOrganics</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Baby Care</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>97.40000000000001</v>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Tier 1 — Premier</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>https://economictimes.indiatimes.com/dabur-tinyorganics-investment</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>P&amp;G and Dabur Announce Joint Venture for Oral Care Products in Southeast Asia</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>CNBC</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>$200 million</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Procter &amp; Gamble and Dabur</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Oral Care</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Southeast Asia</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>82</v>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>92.2</v>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Tier 2 — Reputable</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cnbc.com/pg-dabur-joint-venture-oral-care</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>ITC Acquires Healthy Breakfast Brand MorningStar for ₹1,200 Crore</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>MoneyControl</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>₹1,200 crore (approximately $140 million)</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>MorningStar</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Packaged Foods</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>82</v>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>92.2</v>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Tier 2 — Reputable</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.moneycontrol.com/news/itc-morningstar-acquisition</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Godrej Consumer Products to Acquire African Home Care Brand CleanAfrica</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Business Standard</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>$85 million</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Godrej Consumer Products Limited (GCPL)</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>CleanAfrica</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Household Care</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>82</v>
+      </c>
+      <c r="L15" s="2" t="n">
+        <v>92.2</v>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Tier 2 — Reputable</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.business-standard.com/godrej-cleanafrica-acquisition</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Coca-Cola Acquires Minority Stake in African Juice Brand FreshPressAfrica</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Forbes</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Investment</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed (estimated $50-70 million)</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>The Coca-Cola Company</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>FreshPressAfrica</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Beverages</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>82</v>
+      </c>
+      <c r="L16" s="2" t="n">
+        <v>92.2</v>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Tier 2 — Reputable</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.forbes.com/coca-cola-freshpressafrica-investment</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>General Mills Acquires European Plant-Based Dairy Brand OatLux for $320 Million</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>CNBC</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>$320 million</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>General Mills</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>OatLux</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Dairy Alternatives</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K17" s="3" t="n">
+        <v>82</v>
+      </c>
+      <c r="L17" s="2" t="n">
+        <v>92.2</v>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Tier 2 — Reputable</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cnbc.com/general-mills-oatlux-acquisition</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Ferrero Group Acquires UK Premium Chocolate Brand Thornton &amp; Moore</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>The Guardian</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>£180 million ($225 million) estimated</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Ferrero Group</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Thornton &amp; Moore</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Confectionery</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>82</v>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>92.2</v>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Tier 2 — Reputable</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theguardian.com/business/ferrero-thornton-moore-acquisition</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Colgate-Palmolive Invests in AI-Powered Oral Health Startup SmileTech</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Forbes</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Investment</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>$75 million</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Colgate-Palmolive</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>SmileTech</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Oral Care</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>82</v>
+      </c>
+      <c r="L19" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>Tier 2 — Reputable</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.forbes.com/colgate-smiletech-investment</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Announces ₹2,500 Crore Investment in New Food Processing Plant</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>LiveMint</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Investment</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>₹2,500 crore ($300 million)</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited (HUL)</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Packaged Foods</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="K20" s="3" t="n">
+        <v>82</v>
+      </c>
+      <c r="L20" s="2" t="n">
+        <v>89.8</v>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>Tier 2 — Reputable</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.livemint.com/companies/hul-food-processing-plant</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Church &amp; Dwight Acquires European Laundry Pod Brand FreshPods</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>MarketWatch</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>$120 million</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Church &amp; Dwight Co.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>FreshPods</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Household Care</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K21" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="L21" s="2" t="n">
+        <v>85.40000000000001</v>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>Tier 3 — Niche/Regional</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.marketwatch.com/church-dwight-freshpods</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Kellogg's Acquires Organic Granola Brand NatureCrunch for $95M</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Food Dive</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>$95 million</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Kellogg Company</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>NatureCrunch</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Packaged Foods</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="L22" s="2" t="n">
+        <v>85.40000000000001</v>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>Tier 3 — Niche/Regional</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fooddive.com/kelloggs-naturecrunch-acquisition</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Conagra Brands Acquires Asian Frozen Food Maker WokFresh for $260M</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>$260M</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Conagra Brands</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>WokFresh</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Packaged Foods</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="L23" s="2" t="n">
+        <v>85.40000000000001</v>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>Tier 3 — Niche/Regional</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/news/conagra-wokfresh-acquisition</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N3"/>
+  <autoFilter ref="A1:N23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Two-tier dedup — LLM verification for grey-zone similarity pairs
- Tier 1 (cosine >= 0.80): Auto-merge (high confidence)
- Tier 2 (cosine 0.60-0.80): LLM verifies if same deal event
- Caught the Henkel/Olaplex duplicate at 0.699 similarity
- Uses gpt-4o-mini with YES/NO for minimal cost
</commit_message>
<xml_diff>
--- a/docs/newsletter.xlsx
+++ b/docs/newsletter.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FMCG Deal Intelligence" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FMCG Deal Intelligence'!$A$1:$N$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FMCG Deal Intelligence'!$A$1:$N$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -697,13 +697,13 @@
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>40</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>68.8</v>
+        <v>71.2</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
@@ -713,65 +713,11 @@
       <c r="N4" s="2" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNSThvLUYtMmI5VGN2cHNRRG50c09JZkluZVRqVDluYmt4SEJXUnJVSzVnVDVrbFFpb2tmNlBFVmlqSjcwOWVRdGZoZjFYZnRITHNiYlZuWFpZTTJsUkFSNlhFaHc2QWxONEtQUUROWWRFT2YxTGhpR2FBYlBSUTRROV9zb2RwNkJtUWhkQTQxMlhKRVEzLXYxUnk5U2VTNVUzdTlfNmZuMlg2d2o5TWJ0djZn?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Henkel AG &amp; Co. KGaA (Vz.) stock gains on Olaplex acquisition talks and sustainability push amid CEO - AD HOC NEWS</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>AD HOC NEWS</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>M&amp;A</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Henkel AG &amp; Co. KGaA</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Olaplex</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="K5" s="4" t="n">
-        <v>40</v>
-      </c>
-      <c r="L5" s="2" t="n">
-        <v>62.8</v>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxORDFTLWN0eHI4YTJTUWdOZW55blc3YnlSeWstTFRHWVlBR0duSkFSaHEzaktXSWZTaXp1LTFGOWFrc3NaaUlKWGVNUkpHQndNZFVXSzFfcUQ0WEhNeXF3dzlQSFYwZzRHd0RBemY3WVE0b0N5TzBKZER3NzJGLWZnZ1NlVldMUlFiTUY0WlkxTE5ESVlCNkt1azhXbW04VThhYTFfSk9NR3hZcTZrS0JSQWlXakhHX1JfZ2tKWk51eW9jUQ?oc=5</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N5"/>
+  <autoFilter ref="A1:N4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>